<commit_message>
Adjusting egrid_master.qmd to dynamically call final_formatting script dependent on temporal_res parameter, correcting column names in metric_structure.xlsx, adding comments to final_formatting scripts.
</commit_message>
<xml_diff>
--- a/data/static_tables/metric_structure.xlsx
+++ b/data/static_tables/metric_structure.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\projects\eGrid\production_model\users\gofortht\data\static_tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EB99943-3AA4-4549-A0EE-6B90B4DE5ACF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9BB9FB4-03D0-4599-A2C0-AD596F345934}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="4" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="7" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="unit_annual" sheetId="1" r:id="rId1"/>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12212" uniqueCount="4556">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12212" uniqueCount="4566">
   <si>
     <t>Name</t>
   </si>
@@ -13723,6 +13723,36 @@
   </si>
   <si>
     <t>BAGENABM2</t>
+  </si>
+  <si>
+    <t>STCHGRT2</t>
+  </si>
+  <si>
+    <t>STFSHGRT2</t>
+  </si>
+  <si>
+    <t>BAFSHGRT2</t>
+  </si>
+  <si>
+    <t>BACHGRT2</t>
+  </si>
+  <si>
+    <t>SRFSHGRT2</t>
+  </si>
+  <si>
+    <t>SRCHGRT2</t>
+  </si>
+  <si>
+    <t>NRCHGRT2</t>
+  </si>
+  <si>
+    <t>NRFSHGRT2</t>
+  </si>
+  <si>
+    <t>USCHGRT2</t>
+  </si>
+  <si>
+    <t>USFSHGRT2</t>
   </si>
 </sst>
 </file>
@@ -20715,7 +20745,7 @@
         <v>1645</v>
       </c>
       <c r="B121" s="96" t="s">
-        <v>1646</v>
+        <v>4561</v>
       </c>
       <c r="C121" s="130" t="s">
         <v>201</v>
@@ -20747,7 +20777,7 @@
         <v>1649</v>
       </c>
       <c r="B123" s="96" t="s">
-        <v>1650</v>
+        <v>4560</v>
       </c>
       <c r="C123" s="130" t="s">
         <v>201</v>
@@ -28390,7 +28420,7 @@
         <v>2134</v>
       </c>
       <c r="B121" s="96" t="s">
-        <v>2135</v>
+        <v>4562</v>
       </c>
       <c r="C121" s="130" t="s">
         <v>201</v>
@@ -28422,7 +28452,7 @@
         <v>2138</v>
       </c>
       <c r="B123" s="96" t="s">
-        <v>2139</v>
+        <v>4563</v>
       </c>
       <c r="C123" s="130" t="s">
         <v>201</v>
@@ -36054,7 +36084,7 @@
         <v>2622</v>
       </c>
       <c r="B119" s="96" t="s">
-        <v>2623</v>
+        <v>4564</v>
       </c>
       <c r="C119" s="130" t="s">
         <v>201</v>
@@ -36086,7 +36116,7 @@
         <v>2626</v>
       </c>
       <c r="B121" s="96" t="s">
-        <v>2627</v>
+        <v>4565</v>
       </c>
       <c r="C121" s="130" t="s">
         <v>201</v>
@@ -50847,7 +50877,7 @@
         <v>669</v>
       </c>
       <c r="B121" s="28" t="s">
-        <v>670</v>
+        <v>4556</v>
       </c>
       <c r="C121" s="130" t="s">
         <v>201</v>
@@ -50879,7 +50909,7 @@
         <v>673</v>
       </c>
       <c r="B123" s="28" t="s">
-        <v>674</v>
+        <v>4557</v>
       </c>
       <c r="C123" s="130" t="s">
         <v>201</v>
@@ -58532,7 +58562,7 @@
         <v>1158</v>
       </c>
       <c r="B121" s="96" t="s">
-        <v>1159</v>
+        <v>4559</v>
       </c>
       <c r="C121" s="130" t="s">
         <v>201</v>
@@ -58564,7 +58594,7 @@
         <v>1162</v>
       </c>
       <c r="B123" s="96" t="s">
-        <v>1163</v>
+        <v>4558</v>
       </c>
       <c r="C123" s="130" t="s">
         <v>201</v>
@@ -60652,6 +60682,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="6c854b04-c9c6-4391-adbe-2e73191270e7" xsi:nil="true"/>
@@ -60660,15 +60699,6 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -60932,20 +60962,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CCA6965B-A23A-4F60-9CAE-00FD555BD4D8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7A2EA77E-CA9B-4563-9A5E-2F50B3C8BA13}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="6c854b04-c9c6-4391-adbe-2e73191270e7"/>
     <ds:schemaRef ds:uri="059b9c67-646b-4b4e-9ab1-2b1c805d0390"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CCA6965B-A23A-4F60-9CAE-00FD555BD4D8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>